<commit_message>
update pathway enrichment with new cluster names
</commit_message>
<xml_diff>
--- a/supplementary_tables/SuppTable4_pathway_enrichment.xlsx
+++ b/supplementary_tables/SuppTable4_pathway_enrichment.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="1369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1377" uniqueCount="1377">
   <si>
     <t xml:space="preserve">Cluster</t>
   </si>
@@ -4123,6 +4123,30 @@
   </si>
   <si>
     <t xml:space="preserve">8/25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Th1/Th2 Effector Hyper-Activation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Dysregulated Repair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Effector Cytokine &amp; Chemokine Activation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Exhaustion &amp; Chronic Inflammation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Neuroinflammation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Niche Homeostasis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Neuro-Recovery Failure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Interferons &amp; Cytotoxicity</t>
   </si>
 </sst>
 </file>
@@ -5914,7 +5938,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B12" t="s">
         <v>33</v>
@@ -5943,7 +5967,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B13" t="s">
         <v>33</v>
@@ -5972,7 +5996,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
@@ -6001,7 +6025,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
@@ -6030,7 +6054,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -6059,7 +6083,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B17" t="s">
         <v>10</v>
@@ -6088,7 +6112,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -6117,7 +6141,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B19" t="s">
         <v>33</v>
@@ -6146,7 +6170,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
@@ -6175,7 +6199,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="B21" t="s">
         <v>10</v>
@@ -6929,7 +6953,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="B47" t="s">
         <v>25</v>
@@ -6958,7 +6982,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="B48" t="s">
         <v>33</v>
@@ -6987,7 +7011,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="B49" t="s">
         <v>33</v>
@@ -7016,7 +7040,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="B50" t="s">
         <v>33</v>
@@ -7045,7 +7069,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="B51" t="s">
         <v>33</v>
@@ -7074,7 +7098,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="B52" t="s">
         <v>33</v>
@@ -7143,7 +7167,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -7172,7 +7196,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -7201,7 +7225,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -7230,7 +7254,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
@@ -7259,7 +7283,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
@@ -7288,7 +7312,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
@@ -7317,7 +7341,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
@@ -7346,7 +7370,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
@@ -7375,7 +7399,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B10" t="s">
         <v>33</v>
@@ -7404,7 +7428,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="B11" t="s">
         <v>25</v>
@@ -7433,7 +7457,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="B12" t="s">
         <v>111</v>
@@ -7462,7 +7486,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="B13" t="s">
         <v>33</v>
@@ -7491,7 +7515,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="B14" t="s">
         <v>25</v>
@@ -7520,7 +7544,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="B15" t="s">
         <v>25</v>
@@ -7665,7 +7689,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
@@ -7694,7 +7718,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="B21" t="s">
         <v>33</v>
@@ -7723,7 +7747,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="B22" t="s">
         <v>33</v>
@@ -7752,7 +7776,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="B23" t="s">
         <v>33</v>
@@ -7781,7 +7805,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>272</v>
+        <v>1374</v>
       </c>
       <c r="B24" t="s">
         <v>25</v>
@@ -7810,7 +7834,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B25" t="s">
         <v>33</v>
@@ -7839,7 +7863,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B26" t="s">
         <v>25</v>
@@ -7868,7 +7892,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
@@ -7897,7 +7921,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B28" t="s">
         <v>25</v>
@@ -7926,7 +7950,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B29" t="s">
         <v>25</v>
@@ -7955,7 +7979,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B30" t="s">
         <v>33</v>
@@ -7984,7 +8008,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B31" t="s">
         <v>33</v>
@@ -8013,7 +8037,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B32" t="s">
         <v>25</v>
@@ -8042,7 +8066,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B33" t="s">
         <v>25</v>
@@ -8071,7 +8095,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="B34" t="s">
         <v>25</v>
@@ -8720,7 +8744,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="B22" t="s">
         <v>33</v>
@@ -8749,7 +8773,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="B23" t="s">
         <v>33</v>
@@ -8778,7 +8802,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="B24" t="s">
         <v>33</v>
@@ -8807,7 +8831,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="B25" t="s">
         <v>33</v>
@@ -8836,7 +8860,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="B26" t="s">
         <v>33</v>
@@ -8865,7 +8889,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="B27" t="s">
         <v>111</v>
@@ -14366,7 +14390,7 @@
         <v>352</v>
       </c>
       <c r="B137" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C137" t="s">
         <v>33</v>
@@ -14404,7 +14428,7 @@
         <v>352</v>
       </c>
       <c r="B138" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C138" t="s">
         <v>33</v>
@@ -14442,7 +14466,7 @@
         <v>352</v>
       </c>
       <c r="B139" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C139" t="s">
         <v>33</v>
@@ -14480,7 +14504,7 @@
         <v>352</v>
       </c>
       <c r="B140" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C140" t="s">
         <v>33</v>
@@ -14518,7 +14542,7 @@
         <v>352</v>
       </c>
       <c r="B141" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C141" t="s">
         <v>33</v>
@@ -14556,7 +14580,7 @@
         <v>352</v>
       </c>
       <c r="B142" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C142" t="s">
         <v>111</v>
@@ -14594,7 +14618,7 @@
         <v>352</v>
       </c>
       <c r="B143" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C143" t="s">
         <v>33</v>
@@ -14632,7 +14656,7 @@
         <v>352</v>
       </c>
       <c r="B144" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C144" t="s">
         <v>33</v>
@@ -14670,7 +14694,7 @@
         <v>352</v>
       </c>
       <c r="B145" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C145" t="s">
         <v>25</v>
@@ -14708,7 +14732,7 @@
         <v>352</v>
       </c>
       <c r="B146" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C146" t="s">
         <v>25</v>
@@ -14746,7 +14770,7 @@
         <v>352</v>
       </c>
       <c r="B147" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C147" t="s">
         <v>33</v>
@@ -14784,7 +14808,7 @@
         <v>352</v>
       </c>
       <c r="B148" t="s">
-        <v>317</v>
+        <v>1376</v>
       </c>
       <c r="C148" t="s">
         <v>25</v>
@@ -17254,7 +17278,7 @@
         <v>771</v>
       </c>
       <c r="B213" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C213" t="s">
         <v>33</v>
@@ -17292,7 +17316,7 @@
         <v>771</v>
       </c>
       <c r="B214" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C214" t="s">
         <v>33</v>
@@ -17330,7 +17354,7 @@
         <v>771</v>
       </c>
       <c r="B215" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C215" t="s">
         <v>10</v>
@@ -17368,7 +17392,7 @@
         <v>771</v>
       </c>
       <c r="B216" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C216" t="s">
         <v>33</v>
@@ -17406,7 +17430,7 @@
         <v>771</v>
       </c>
       <c r="B217" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C217" t="s">
         <v>10</v>
@@ -17444,7 +17468,7 @@
         <v>771</v>
       </c>
       <c r="B218" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C218" t="s">
         <v>10</v>
@@ -17482,7 +17506,7 @@
         <v>771</v>
       </c>
       <c r="B219" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C219" t="s">
         <v>10</v>
@@ -17520,7 +17544,7 @@
         <v>771</v>
       </c>
       <c r="B220" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C220" t="s">
         <v>33</v>
@@ -17558,7 +17582,7 @@
         <v>771</v>
       </c>
       <c r="B221" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C221" t="s">
         <v>33</v>
@@ -17596,7 +17620,7 @@
         <v>771</v>
       </c>
       <c r="B222" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C222" t="s">
         <v>10</v>
@@ -17634,7 +17658,7 @@
         <v>771</v>
       </c>
       <c r="B223" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C223" t="s">
         <v>10</v>
@@ -17672,7 +17696,7 @@
         <v>771</v>
       </c>
       <c r="B224" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C224" t="s">
         <v>10</v>
@@ -17710,7 +17734,7 @@
         <v>771</v>
       </c>
       <c r="B225" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C225" t="s">
         <v>10</v>
@@ -17748,7 +17772,7 @@
         <v>771</v>
       </c>
       <c r="B226" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C226" t="s">
         <v>10</v>
@@ -17786,7 +17810,7 @@
         <v>771</v>
       </c>
       <c r="B227" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C227" t="s">
         <v>10</v>
@@ -17824,7 +17848,7 @@
         <v>771</v>
       </c>
       <c r="B228" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C228" t="s">
         <v>10</v>
@@ -17862,7 +17886,7 @@
         <v>771</v>
       </c>
       <c r="B229" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C229" t="s">
         <v>10</v>
@@ -17900,7 +17924,7 @@
         <v>771</v>
       </c>
       <c r="B230" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C230" t="s">
         <v>10</v>
@@ -17938,7 +17962,7 @@
         <v>771</v>
       </c>
       <c r="B231" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C231" t="s">
         <v>10</v>
@@ -17976,7 +18000,7 @@
         <v>771</v>
       </c>
       <c r="B232" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C232" t="s">
         <v>10</v>
@@ -18014,7 +18038,7 @@
         <v>771</v>
       </c>
       <c r="B233" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C233" t="s">
         <v>10</v>
@@ -18052,7 +18076,7 @@
         <v>771</v>
       </c>
       <c r="B234" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C234" t="s">
         <v>10</v>
@@ -18090,7 +18114,7 @@
         <v>771</v>
       </c>
       <c r="B235" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C235" t="s">
         <v>10</v>
@@ -18128,7 +18152,7 @@
         <v>771</v>
       </c>
       <c r="B236" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C236" t="s">
         <v>10</v>
@@ -18166,7 +18190,7 @@
         <v>771</v>
       </c>
       <c r="B237" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C237" t="s">
         <v>10</v>
@@ -18204,7 +18228,7 @@
         <v>771</v>
       </c>
       <c r="B238" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C238" t="s">
         <v>10</v>
@@ -18242,7 +18266,7 @@
         <v>771</v>
       </c>
       <c r="B239" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C239" t="s">
         <v>10</v>
@@ -18280,7 +18304,7 @@
         <v>771</v>
       </c>
       <c r="B240" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C240" t="s">
         <v>33</v>
@@ -18318,7 +18342,7 @@
         <v>771</v>
       </c>
       <c r="B241" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C241" t="s">
         <v>33</v>
@@ -18356,7 +18380,7 @@
         <v>771</v>
       </c>
       <c r="B242" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C242" t="s">
         <v>10</v>
@@ -18394,7 +18418,7 @@
         <v>771</v>
       </c>
       <c r="B243" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C243" t="s">
         <v>10</v>
@@ -18432,7 +18456,7 @@
         <v>771</v>
       </c>
       <c r="B244" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C244" t="s">
         <v>10</v>
@@ -18470,7 +18494,7 @@
         <v>771</v>
       </c>
       <c r="B245" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C245" t="s">
         <v>10</v>
@@ -18508,7 +18532,7 @@
         <v>771</v>
       </c>
       <c r="B246" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C246" t="s">
         <v>10</v>
@@ -18546,7 +18570,7 @@
         <v>771</v>
       </c>
       <c r="B247" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C247" t="s">
         <v>10</v>
@@ -18584,7 +18608,7 @@
         <v>771</v>
       </c>
       <c r="B248" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C248" t="s">
         <v>10</v>
@@ -18622,7 +18646,7 @@
         <v>771</v>
       </c>
       <c r="B249" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C249" t="s">
         <v>33</v>
@@ -18660,7 +18684,7 @@
         <v>771</v>
       </c>
       <c r="B250" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C250" t="s">
         <v>10</v>
@@ -18698,7 +18722,7 @@
         <v>771</v>
       </c>
       <c r="B251" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C251" t="s">
         <v>10</v>
@@ -18736,7 +18760,7 @@
         <v>771</v>
       </c>
       <c r="B252" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C252" t="s">
         <v>10</v>
@@ -18774,7 +18798,7 @@
         <v>771</v>
       </c>
       <c r="B253" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C253" t="s">
         <v>10</v>
@@ -18812,7 +18836,7 @@
         <v>771</v>
       </c>
       <c r="B254" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C254" t="s">
         <v>33</v>
@@ -18850,7 +18874,7 @@
         <v>771</v>
       </c>
       <c r="B255" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C255" t="s">
         <v>10</v>
@@ -18888,7 +18912,7 @@
         <v>771</v>
       </c>
       <c r="B256" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C256" t="s">
         <v>10</v>
@@ -18926,7 +18950,7 @@
         <v>771</v>
       </c>
       <c r="B257" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C257" t="s">
         <v>10</v>
@@ -18964,7 +18988,7 @@
         <v>771</v>
       </c>
       <c r="B258" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C258" t="s">
         <v>10</v>
@@ -19002,7 +19026,7 @@
         <v>771</v>
       </c>
       <c r="B259" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C259" t="s">
         <v>33</v>
@@ -19040,7 +19064,7 @@
         <v>771</v>
       </c>
       <c r="B260" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C260" t="s">
         <v>10</v>
@@ -19078,7 +19102,7 @@
         <v>771</v>
       </c>
       <c r="B261" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C261" t="s">
         <v>10</v>
@@ -19116,7 +19140,7 @@
         <v>771</v>
       </c>
       <c r="B262" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C262" t="s">
         <v>25</v>
@@ -19154,7 +19178,7 @@
         <v>771</v>
       </c>
       <c r="B263" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C263" t="s">
         <v>10</v>
@@ -19192,7 +19216,7 @@
         <v>771</v>
       </c>
       <c r="B264" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C264" t="s">
         <v>10</v>
@@ -19230,7 +19254,7 @@
         <v>771</v>
       </c>
       <c r="B265" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C265" t="s">
         <v>10</v>
@@ -19268,7 +19292,7 @@
         <v>771</v>
       </c>
       <c r="B266" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C266" t="s">
         <v>10</v>
@@ -19306,7 +19330,7 @@
         <v>771</v>
       </c>
       <c r="B267" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C267" t="s">
         <v>33</v>
@@ -19344,7 +19368,7 @@
         <v>771</v>
       </c>
       <c r="B268" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C268" t="s">
         <v>10</v>
@@ -19382,7 +19406,7 @@
         <v>771</v>
       </c>
       <c r="B269" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C269" t="s">
         <v>33</v>
@@ -19420,7 +19444,7 @@
         <v>771</v>
       </c>
       <c r="B270" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C270" t="s">
         <v>33</v>
@@ -19458,7 +19482,7 @@
         <v>771</v>
       </c>
       <c r="B271" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C271" t="s">
         <v>10</v>
@@ -19496,7 +19520,7 @@
         <v>771</v>
       </c>
       <c r="B272" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C272" t="s">
         <v>10</v>
@@ -19534,7 +19558,7 @@
         <v>771</v>
       </c>
       <c r="B273" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C273" t="s">
         <v>10</v>
@@ -19572,7 +19596,7 @@
         <v>771</v>
       </c>
       <c r="B274" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C274" t="s">
         <v>10</v>
@@ -19610,7 +19634,7 @@
         <v>771</v>
       </c>
       <c r="B275" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C275" t="s">
         <v>10</v>
@@ -19648,7 +19672,7 @@
         <v>771</v>
       </c>
       <c r="B276" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C276" t="s">
         <v>10</v>
@@ -19686,7 +19710,7 @@
         <v>771</v>
       </c>
       <c r="B277" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C277" t="s">
         <v>10</v>
@@ -19724,7 +19748,7 @@
         <v>771</v>
       </c>
       <c r="B278" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C278" t="s">
         <v>10</v>
@@ -19762,7 +19786,7 @@
         <v>771</v>
       </c>
       <c r="B279" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C279" t="s">
         <v>10</v>
@@ -19800,7 +19824,7 @@
         <v>771</v>
       </c>
       <c r="B280" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C280" t="s">
         <v>10</v>
@@ -19838,7 +19862,7 @@
         <v>771</v>
       </c>
       <c r="B281" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C281" t="s">
         <v>10</v>
@@ -19876,7 +19900,7 @@
         <v>771</v>
       </c>
       <c r="B282" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C282" t="s">
         <v>10</v>
@@ -19914,7 +19938,7 @@
         <v>771</v>
       </c>
       <c r="B283" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C283" t="s">
         <v>10</v>
@@ -19952,7 +19976,7 @@
         <v>771</v>
       </c>
       <c r="B284" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C284" t="s">
         <v>10</v>
@@ -19990,7 +20014,7 @@
         <v>771</v>
       </c>
       <c r="B285" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C285" t="s">
         <v>10</v>
@@ -20028,7 +20052,7 @@
         <v>771</v>
       </c>
       <c r="B286" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C286" t="s">
         <v>10</v>
@@ -20066,7 +20090,7 @@
         <v>771</v>
       </c>
       <c r="B287" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C287" t="s">
         <v>10</v>
@@ -20104,7 +20128,7 @@
         <v>771</v>
       </c>
       <c r="B288" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C288" t="s">
         <v>10</v>
@@ -20142,7 +20166,7 @@
         <v>771</v>
       </c>
       <c r="B289" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C289" t="s">
         <v>10</v>
@@ -20180,7 +20204,7 @@
         <v>771</v>
       </c>
       <c r="B290" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C290" t="s">
         <v>10</v>
@@ -20218,7 +20242,7 @@
         <v>771</v>
       </c>
       <c r="B291" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C291" t="s">
         <v>10</v>
@@ -20256,7 +20280,7 @@
         <v>771</v>
       </c>
       <c r="B292" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C292" t="s">
         <v>10</v>
@@ -20294,7 +20318,7 @@
         <v>771</v>
       </c>
       <c r="B293" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C293" t="s">
         <v>10</v>
@@ -20332,7 +20356,7 @@
         <v>771</v>
       </c>
       <c r="B294" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C294" t="s">
         <v>10</v>
@@ -20370,7 +20394,7 @@
         <v>771</v>
       </c>
       <c r="B295" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C295" t="s">
         <v>10</v>
@@ -20408,7 +20432,7 @@
         <v>771</v>
       </c>
       <c r="B296" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C296" t="s">
         <v>10</v>
@@ -20446,7 +20470,7 @@
         <v>771</v>
       </c>
       <c r="B297" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C297" t="s">
         <v>33</v>
@@ -20484,7 +20508,7 @@
         <v>771</v>
       </c>
       <c r="B298" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C298" t="s">
         <v>33</v>
@@ -20522,7 +20546,7 @@
         <v>771</v>
       </c>
       <c r="B299" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C299" t="s">
         <v>33</v>
@@ -20560,7 +20584,7 @@
         <v>771</v>
       </c>
       <c r="B300" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C300" t="s">
         <v>10</v>
@@ -20598,7 +20622,7 @@
         <v>771</v>
       </c>
       <c r="B301" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C301" t="s">
         <v>10</v>
@@ -20636,7 +20660,7 @@
         <v>771</v>
       </c>
       <c r="B302" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C302" t="s">
         <v>10</v>
@@ -20674,7 +20698,7 @@
         <v>771</v>
       </c>
       <c r="B303" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C303" t="s">
         <v>10</v>
@@ -20712,7 +20736,7 @@
         <v>771</v>
       </c>
       <c r="B304" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C304" t="s">
         <v>10</v>
@@ -20750,7 +20774,7 @@
         <v>771</v>
       </c>
       <c r="B305" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C305" t="s">
         <v>10</v>
@@ -20788,7 +20812,7 @@
         <v>771</v>
       </c>
       <c r="B306" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C306" t="s">
         <v>10</v>
@@ -20826,7 +20850,7 @@
         <v>771</v>
       </c>
       <c r="B307" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C307" t="s">
         <v>10</v>
@@ -20864,7 +20888,7 @@
         <v>771</v>
       </c>
       <c r="B308" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C308" t="s">
         <v>25</v>
@@ -20902,7 +20926,7 @@
         <v>771</v>
       </c>
       <c r="B309" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C309" t="s">
         <v>10</v>
@@ -20940,7 +20964,7 @@
         <v>771</v>
       </c>
       <c r="B310" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C310" t="s">
         <v>10</v>
@@ -20978,7 +21002,7 @@
         <v>771</v>
       </c>
       <c r="B311" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C311" t="s">
         <v>10</v>
@@ -21016,7 +21040,7 @@
         <v>771</v>
       </c>
       <c r="B312" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C312" t="s">
         <v>10</v>
@@ -21054,7 +21078,7 @@
         <v>771</v>
       </c>
       <c r="B313" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C313" t="s">
         <v>33</v>
@@ -21092,7 +21116,7 @@
         <v>771</v>
       </c>
       <c r="B314" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C314" t="s">
         <v>33</v>
@@ -21130,7 +21154,7 @@
         <v>771</v>
       </c>
       <c r="B315" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C315" t="s">
         <v>33</v>
@@ -21168,7 +21192,7 @@
         <v>771</v>
       </c>
       <c r="B316" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C316" t="s">
         <v>10</v>
@@ -21206,7 +21230,7 @@
         <v>771</v>
       </c>
       <c r="B317" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C317" t="s">
         <v>10</v>
@@ -21244,7 +21268,7 @@
         <v>771</v>
       </c>
       <c r="B318" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C318" t="s">
         <v>33</v>
@@ -21282,7 +21306,7 @@
         <v>771</v>
       </c>
       <c r="B319" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C319" t="s">
         <v>10</v>
@@ -21320,7 +21344,7 @@
         <v>771</v>
       </c>
       <c r="B320" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C320" t="s">
         <v>10</v>
@@ -21358,7 +21382,7 @@
         <v>771</v>
       </c>
       <c r="B321" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C321" t="s">
         <v>10</v>
@@ -21396,7 +21420,7 @@
         <v>771</v>
       </c>
       <c r="B322" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C322" t="s">
         <v>10</v>
@@ -21434,7 +21458,7 @@
         <v>771</v>
       </c>
       <c r="B323" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C323" t="s">
         <v>33</v>
@@ -21472,7 +21496,7 @@
         <v>771</v>
       </c>
       <c r="B324" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C324" t="s">
         <v>33</v>
@@ -21510,7 +21534,7 @@
         <v>771</v>
       </c>
       <c r="B325" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C325" t="s">
         <v>33</v>
@@ -21548,7 +21572,7 @@
         <v>771</v>
       </c>
       <c r="B326" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C326" t="s">
         <v>33</v>
@@ -21586,7 +21610,7 @@
         <v>771</v>
       </c>
       <c r="B327" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C327" t="s">
         <v>10</v>
@@ -21624,7 +21648,7 @@
         <v>771</v>
       </c>
       <c r="B328" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C328" t="s">
         <v>10</v>
@@ -21662,7 +21686,7 @@
         <v>771</v>
       </c>
       <c r="B329" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C329" t="s">
         <v>10</v>
@@ -21700,7 +21724,7 @@
         <v>771</v>
       </c>
       <c r="B330" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C330" t="s">
         <v>10</v>
@@ -21738,7 +21762,7 @@
         <v>771</v>
       </c>
       <c r="B331" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C331" t="s">
         <v>10</v>
@@ -21776,7 +21800,7 @@
         <v>771</v>
       </c>
       <c r="B332" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C332" t="s">
         <v>10</v>
@@ -21814,7 +21838,7 @@
         <v>771</v>
       </c>
       <c r="B333" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C333" t="s">
         <v>10</v>
@@ -21852,7 +21876,7 @@
         <v>771</v>
       </c>
       <c r="B334" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C334" t="s">
         <v>10</v>
@@ -21890,7 +21914,7 @@
         <v>771</v>
       </c>
       <c r="B335" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C335" t="s">
         <v>10</v>
@@ -21928,7 +21952,7 @@
         <v>771</v>
       </c>
       <c r="B336" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C336" t="s">
         <v>10</v>
@@ -21966,7 +21990,7 @@
         <v>771</v>
       </c>
       <c r="B337" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C337" t="s">
         <v>10</v>
@@ -22004,7 +22028,7 @@
         <v>771</v>
       </c>
       <c r="B338" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C338" t="s">
         <v>10</v>
@@ -22042,7 +22066,7 @@
         <v>771</v>
       </c>
       <c r="B339" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C339" t="s">
         <v>10</v>
@@ -22080,7 +22104,7 @@
         <v>771</v>
       </c>
       <c r="B340" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C340" t="s">
         <v>10</v>
@@ -22118,7 +22142,7 @@
         <v>771</v>
       </c>
       <c r="B341" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C341" t="s">
         <v>10</v>
@@ -22156,7 +22180,7 @@
         <v>771</v>
       </c>
       <c r="B342" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C342" t="s">
         <v>10</v>
@@ -22194,7 +22218,7 @@
         <v>771</v>
       </c>
       <c r="B343" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C343" t="s">
         <v>10</v>
@@ -22232,7 +22256,7 @@
         <v>771</v>
       </c>
       <c r="B344" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C344" t="s">
         <v>10</v>
@@ -22270,7 +22294,7 @@
         <v>771</v>
       </c>
       <c r="B345" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C345" t="s">
         <v>10</v>
@@ -22308,7 +22332,7 @@
         <v>771</v>
       </c>
       <c r="B346" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C346" t="s">
         <v>10</v>
@@ -22346,7 +22370,7 @@
         <v>771</v>
       </c>
       <c r="B347" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C347" t="s">
         <v>33</v>
@@ -22384,7 +22408,7 @@
         <v>771</v>
       </c>
       <c r="B348" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C348" t="s">
         <v>33</v>
@@ -22422,7 +22446,7 @@
         <v>771</v>
       </c>
       <c r="B349" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C349" t="s">
         <v>33</v>
@@ -22460,7 +22484,7 @@
         <v>771</v>
       </c>
       <c r="B350" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C350" t="s">
         <v>33</v>
@@ -22498,7 +22522,7 @@
         <v>771</v>
       </c>
       <c r="B351" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C351" t="s">
         <v>33</v>
@@ -22536,7 +22560,7 @@
         <v>771</v>
       </c>
       <c r="B352" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C352" t="s">
         <v>33</v>
@@ -22574,7 +22598,7 @@
         <v>771</v>
       </c>
       <c r="B353" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C353" t="s">
         <v>33</v>
@@ -22612,7 +22636,7 @@
         <v>771</v>
       </c>
       <c r="B354" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C354" t="s">
         <v>33</v>
@@ -22650,7 +22674,7 @@
         <v>771</v>
       </c>
       <c r="B355" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C355" t="s">
         <v>33</v>
@@ -22688,7 +22712,7 @@
         <v>771</v>
       </c>
       <c r="B356" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C356" t="s">
         <v>33</v>
@@ -22726,7 +22750,7 @@
         <v>771</v>
       </c>
       <c r="B357" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C357" t="s">
         <v>33</v>
@@ -22764,7 +22788,7 @@
         <v>771</v>
       </c>
       <c r="B358" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C358" t="s">
         <v>33</v>
@@ -22802,7 +22826,7 @@
         <v>771</v>
       </c>
       <c r="B359" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C359" t="s">
         <v>33</v>
@@ -22840,7 +22864,7 @@
         <v>771</v>
       </c>
       <c r="B360" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C360" t="s">
         <v>33</v>
@@ -22878,7 +22902,7 @@
         <v>771</v>
       </c>
       <c r="B361" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C361" t="s">
         <v>25</v>
@@ -22916,7 +22940,7 @@
         <v>771</v>
       </c>
       <c r="B362" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C362" t="s">
         <v>33</v>
@@ -22954,7 +22978,7 @@
         <v>771</v>
       </c>
       <c r="B363" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C363" t="s">
         <v>33</v>
@@ -22992,7 +23016,7 @@
         <v>771</v>
       </c>
       <c r="B364" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C364" t="s">
         <v>25</v>
@@ -23030,7 +23054,7 @@
         <v>771</v>
       </c>
       <c r="B365" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C365" t="s">
         <v>33</v>
@@ -23068,7 +23092,7 @@
         <v>771</v>
       </c>
       <c r="B366" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C366" t="s">
         <v>33</v>
@@ -23106,7 +23130,7 @@
         <v>771</v>
       </c>
       <c r="B367" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C367" t="s">
         <v>33</v>
@@ -23144,7 +23168,7 @@
         <v>771</v>
       </c>
       <c r="B368" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C368" t="s">
         <v>25</v>
@@ -23182,7 +23206,7 @@
         <v>771</v>
       </c>
       <c r="B369" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C369" t="s">
         <v>33</v>
@@ -23220,7 +23244,7 @@
         <v>771</v>
       </c>
       <c r="B370" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C370" t="s">
         <v>33</v>
@@ -23258,7 +23282,7 @@
         <v>771</v>
       </c>
       <c r="B371" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C371" t="s">
         <v>33</v>
@@ -23296,7 +23320,7 @@
         <v>771</v>
       </c>
       <c r="B372" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C372" t="s">
         <v>25</v>
@@ -23334,7 +23358,7 @@
         <v>771</v>
       </c>
       <c r="B373" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C373" t="s">
         <v>33</v>
@@ -23372,7 +23396,7 @@
         <v>771</v>
       </c>
       <c r="B374" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C374" t="s">
         <v>25</v>
@@ -23410,7 +23434,7 @@
         <v>771</v>
       </c>
       <c r="B375" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C375" t="s">
         <v>33</v>
@@ -23448,7 +23472,7 @@
         <v>771</v>
       </c>
       <c r="B376" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C376" t="s">
         <v>111</v>
@@ -23486,7 +23510,7 @@
         <v>771</v>
       </c>
       <c r="B377" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C377" t="s">
         <v>25</v>
@@ -23524,7 +23548,7 @@
         <v>771</v>
       </c>
       <c r="B378" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C378" t="s">
         <v>33</v>
@@ -23562,7 +23586,7 @@
         <v>771</v>
       </c>
       <c r="B379" t="s">
-        <v>138</v>
+        <v>1369</v>
       </c>
       <c r="C379" t="s">
         <v>33</v>
@@ -25766,7 +25790,7 @@
         <v>771</v>
       </c>
       <c r="B437" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C437" t="s">
         <v>25</v>
@@ -25804,7 +25828,7 @@
         <v>771</v>
       </c>
       <c r="B438" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C438" t="s">
         <v>33</v>
@@ -25842,7 +25866,7 @@
         <v>771</v>
       </c>
       <c r="B439" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C439" t="s">
         <v>33</v>
@@ -25880,7 +25904,7 @@
         <v>771</v>
       </c>
       <c r="B440" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C440" t="s">
         <v>33</v>
@@ -25918,7 +25942,7 @@
         <v>771</v>
       </c>
       <c r="B441" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C441" t="s">
         <v>33</v>
@@ -25956,7 +25980,7 @@
         <v>771</v>
       </c>
       <c r="B442" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C442" t="s">
         <v>33</v>
@@ -25994,7 +26018,7 @@
         <v>771</v>
       </c>
       <c r="B443" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C443" t="s">
         <v>33</v>
@@ -26032,7 +26056,7 @@
         <v>771</v>
       </c>
       <c r="B444" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C444" t="s">
         <v>33</v>
@@ -26070,7 +26094,7 @@
         <v>771</v>
       </c>
       <c r="B445" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C445" t="s">
         <v>33</v>
@@ -26108,7 +26132,7 @@
         <v>771</v>
       </c>
       <c r="B446" t="s">
-        <v>206</v>
+        <v>1370</v>
       </c>
       <c r="C446" t="s">
         <v>33</v>
@@ -26146,7 +26170,7 @@
         <v>1169</v>
       </c>
       <c r="B447" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C447" t="s">
         <v>10</v>
@@ -26184,7 +26208,7 @@
         <v>1169</v>
       </c>
       <c r="B448" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C448" t="s">
         <v>33</v>
@@ -26222,7 +26246,7 @@
         <v>1169</v>
       </c>
       <c r="B449" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C449" t="s">
         <v>10</v>
@@ -26260,7 +26284,7 @@
         <v>1169</v>
       </c>
       <c r="B450" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C450" t="s">
         <v>10</v>
@@ -26298,7 +26322,7 @@
         <v>1169</v>
       </c>
       <c r="B451" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C451" t="s">
         <v>10</v>
@@ -26336,7 +26360,7 @@
         <v>1169</v>
       </c>
       <c r="B452" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C452" t="s">
         <v>10</v>
@@ -26374,7 +26398,7 @@
         <v>1169</v>
       </c>
       <c r="B453" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C453" t="s">
         <v>10</v>
@@ -26412,7 +26436,7 @@
         <v>1169</v>
       </c>
       <c r="B454" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C454" t="s">
         <v>10</v>
@@ -26450,7 +26474,7 @@
         <v>1169</v>
       </c>
       <c r="B455" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C455" t="s">
         <v>33</v>
@@ -26488,7 +26512,7 @@
         <v>1169</v>
       </c>
       <c r="B456" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C456" t="s">
         <v>25</v>
@@ -26526,7 +26550,7 @@
         <v>1169</v>
       </c>
       <c r="B457" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C457" t="s">
         <v>33</v>
@@ -26564,7 +26588,7 @@
         <v>1169</v>
       </c>
       <c r="B458" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C458" t="s">
         <v>33</v>
@@ -26602,7 +26626,7 @@
         <v>1169</v>
       </c>
       <c r="B459" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C459" t="s">
         <v>10</v>
@@ -26640,7 +26664,7 @@
         <v>1169</v>
       </c>
       <c r="B460" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C460" t="s">
         <v>10</v>
@@ -26678,7 +26702,7 @@
         <v>1169</v>
       </c>
       <c r="B461" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C461" t="s">
         <v>10</v>
@@ -26716,7 +26740,7 @@
         <v>1169</v>
       </c>
       <c r="B462" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C462" t="s">
         <v>10</v>
@@ -26754,7 +26778,7 @@
         <v>1169</v>
       </c>
       <c r="B463" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C463" t="s">
         <v>10</v>
@@ -26792,7 +26816,7 @@
         <v>1169</v>
       </c>
       <c r="B464" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C464" t="s">
         <v>17</v>
@@ -26830,7 +26854,7 @@
         <v>1169</v>
       </c>
       <c r="B465" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C465" t="s">
         <v>33</v>
@@ -26868,7 +26892,7 @@
         <v>1169</v>
       </c>
       <c r="B466" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C466" t="s">
         <v>25</v>
@@ -26906,7 +26930,7 @@
         <v>1169</v>
       </c>
       <c r="B467" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C467" t="s">
         <v>33</v>
@@ -26944,7 +26968,7 @@
         <v>1169</v>
       </c>
       <c r="B468" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C468" t="s">
         <v>25</v>
@@ -26982,7 +27006,7 @@
         <v>1169</v>
       </c>
       <c r="B469" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C469" t="s">
         <v>25</v>
@@ -27020,7 +27044,7 @@
         <v>1169</v>
       </c>
       <c r="B470" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C470" t="s">
         <v>25</v>
@@ -27058,7 +27082,7 @@
         <v>1169</v>
       </c>
       <c r="B471" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C471" t="s">
         <v>33</v>
@@ -27096,7 +27120,7 @@
         <v>1169</v>
       </c>
       <c r="B472" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C472" t="s">
         <v>33</v>
@@ -27134,7 +27158,7 @@
         <v>1169</v>
       </c>
       <c r="B473" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C473" t="s">
         <v>25</v>
@@ -27172,7 +27196,7 @@
         <v>1169</v>
       </c>
       <c r="B474" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C474" t="s">
         <v>25</v>
@@ -27210,7 +27234,7 @@
         <v>1169</v>
       </c>
       <c r="B475" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C475" t="s">
         <v>25</v>
@@ -27248,7 +27272,7 @@
         <v>1169</v>
       </c>
       <c r="B476" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C476" t="s">
         <v>25</v>
@@ -27286,7 +27310,7 @@
         <v>1169</v>
       </c>
       <c r="B477" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C477" t="s">
         <v>33</v>
@@ -27324,7 +27348,7 @@
         <v>1169</v>
       </c>
       <c r="B478" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C478" t="s">
         <v>25</v>
@@ -27362,7 +27386,7 @@
         <v>1169</v>
       </c>
       <c r="B479" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C479" t="s">
         <v>25</v>
@@ -27400,7 +27424,7 @@
         <v>1169</v>
       </c>
       <c r="B480" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C480" t="s">
         <v>25</v>
@@ -27438,7 +27462,7 @@
         <v>1169</v>
       </c>
       <c r="B481" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C481" t="s">
         <v>25</v>
@@ -27476,7 +27500,7 @@
         <v>1169</v>
       </c>
       <c r="B482" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C482" t="s">
         <v>33</v>
@@ -27514,7 +27538,7 @@
         <v>1169</v>
       </c>
       <c r="B483" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C483" t="s">
         <v>111</v>
@@ -27552,7 +27576,7 @@
         <v>1169</v>
       </c>
       <c r="B484" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C484" t="s">
         <v>33</v>
@@ -27590,7 +27614,7 @@
         <v>1169</v>
       </c>
       <c r="B485" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C485" t="s">
         <v>33</v>
@@ -27628,7 +27652,7 @@
         <v>1169</v>
       </c>
       <c r="B486" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C486" t="s">
         <v>33</v>
@@ -27666,7 +27690,7 @@
         <v>1169</v>
       </c>
       <c r="B487" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C487" t="s">
         <v>33</v>
@@ -27704,7 +27728,7 @@
         <v>1169</v>
       </c>
       <c r="B488" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C488" t="s">
         <v>33</v>
@@ -27742,7 +27766,7 @@
         <v>1169</v>
       </c>
       <c r="B489" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C489" t="s">
         <v>33</v>
@@ -27780,7 +27804,7 @@
         <v>1169</v>
       </c>
       <c r="B490" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C490" t="s">
         <v>25</v>
@@ -27818,7 +27842,7 @@
         <v>1169</v>
       </c>
       <c r="B491" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C491" t="s">
         <v>25</v>
@@ -27856,7 +27880,7 @@
         <v>1169</v>
       </c>
       <c r="B492" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C492" t="s">
         <v>33</v>
@@ -27894,7 +27918,7 @@
         <v>1169</v>
       </c>
       <c r="B493" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C493" t="s">
         <v>33</v>
@@ -27932,7 +27956,7 @@
         <v>1169</v>
       </c>
       <c r="B494" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C494" t="s">
         <v>25</v>
@@ -27970,7 +27994,7 @@
         <v>1169</v>
       </c>
       <c r="B495" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C495" t="s">
         <v>111</v>
@@ -28008,7 +28032,7 @@
         <v>1169</v>
       </c>
       <c r="B496" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C496" t="s">
         <v>33</v>
@@ -28046,7 +28070,7 @@
         <v>1169</v>
       </c>
       <c r="B497" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C497" t="s">
         <v>33</v>
@@ -28084,7 +28108,7 @@
         <v>1169</v>
       </c>
       <c r="B498" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C498" t="s">
         <v>33</v>
@@ -28122,7 +28146,7 @@
         <v>1169</v>
       </c>
       <c r="B499" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C499" t="s">
         <v>33</v>
@@ -28160,7 +28184,7 @@
         <v>1169</v>
       </c>
       <c r="B500" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C500" t="s">
         <v>111</v>
@@ -28198,7 +28222,7 @@
         <v>1169</v>
       </c>
       <c r="B501" t="s">
-        <v>221</v>
+        <v>1371</v>
       </c>
       <c r="C501" t="s">
         <v>33</v>
@@ -28236,7 +28260,7 @@
         <v>1169</v>
       </c>
       <c r="B502" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C502" t="s">
         <v>111</v>
@@ -28274,7 +28298,7 @@
         <v>1169</v>
       </c>
       <c r="B503" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C503" t="s">
         <v>33</v>
@@ -28312,7 +28336,7 @@
         <v>1169</v>
       </c>
       <c r="B504" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C504" t="s">
         <v>25</v>
@@ -28350,7 +28374,7 @@
         <v>1169</v>
       </c>
       <c r="B505" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C505" t="s">
         <v>25</v>
@@ -28388,7 +28412,7 @@
         <v>1169</v>
       </c>
       <c r="B506" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C506" t="s">
         <v>33</v>
@@ -28426,7 +28450,7 @@
         <v>1169</v>
       </c>
       <c r="B507" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C507" t="s">
         <v>111</v>
@@ -28464,7 +28488,7 @@
         <v>1169</v>
       </c>
       <c r="B508" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C508" t="s">
         <v>25</v>
@@ -28502,7 +28526,7 @@
         <v>1169</v>
       </c>
       <c r="B509" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C509" t="s">
         <v>25</v>
@@ -28540,7 +28564,7 @@
         <v>1169</v>
       </c>
       <c r="B510" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C510" t="s">
         <v>25</v>
@@ -28578,7 +28602,7 @@
         <v>1169</v>
       </c>
       <c r="B511" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C511" t="s">
         <v>25</v>
@@ -28616,7 +28640,7 @@
         <v>1169</v>
       </c>
       <c r="B512" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C512" t="s">
         <v>33</v>
@@ -28654,7 +28678,7 @@
         <v>1169</v>
       </c>
       <c r="B513" t="s">
-        <v>242</v>
+        <v>1372</v>
       </c>
       <c r="C513" t="s">
         <v>33</v>
@@ -28996,7 +29020,7 @@
         <v>1169</v>
       </c>
       <c r="B522" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C522" t="s">
         <v>33</v>
@@ -29034,7 +29058,7 @@
         <v>1169</v>
       </c>
       <c r="B523" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C523" t="s">
         <v>33</v>
@@ -29072,7 +29096,7 @@
         <v>1169</v>
       </c>
       <c r="B524" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C524" t="s">
         <v>33</v>
@@ -29110,7 +29134,7 @@
         <v>1169</v>
       </c>
       <c r="B525" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C525" t="s">
         <v>33</v>
@@ -29148,7 +29172,7 @@
         <v>1169</v>
       </c>
       <c r="B526" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C526" t="s">
         <v>33</v>
@@ -29186,7 +29210,7 @@
         <v>1169</v>
       </c>
       <c r="B527" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C527" t="s">
         <v>111</v>
@@ -29224,7 +29248,7 @@
         <v>1169</v>
       </c>
       <c r="B528" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C528" t="s">
         <v>33</v>
@@ -29262,7 +29286,7 @@
         <v>1169</v>
       </c>
       <c r="B529" t="s">
-        <v>263</v>
+        <v>1373</v>
       </c>
       <c r="C529" t="s">
         <v>33</v>
@@ -29300,7 +29324,7 @@
         <v>1169</v>
       </c>
       <c r="B530" t="s">
-        <v>272</v>
+        <v>1374</v>
       </c>
       <c r="C530" t="s">
         <v>25</v>
@@ -29338,7 +29362,7 @@
         <v>1169</v>
       </c>
       <c r="B531" t="s">
-        <v>272</v>
+        <v>1374</v>
       </c>
       <c r="C531" t="s">
         <v>33</v>
@@ -29376,7 +29400,7 @@
         <v>1169</v>
       </c>
       <c r="B532" t="s">
-        <v>272</v>
+        <v>1374</v>
       </c>
       <c r="C532" t="s">
         <v>25</v>
@@ -29414,7 +29438,7 @@
         <v>1169</v>
       </c>
       <c r="B533" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C533" t="s">
         <v>33</v>
@@ -29452,7 +29476,7 @@
         <v>1169</v>
       </c>
       <c r="B534" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C534" t="s">
         <v>25</v>
@@ -29490,7 +29514,7 @@
         <v>1169</v>
       </c>
       <c r="B535" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C535" t="s">
         <v>33</v>
@@ -29528,7 +29552,7 @@
         <v>1169</v>
       </c>
       <c r="B536" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C536" t="s">
         <v>25</v>
@@ -29566,7 +29590,7 @@
         <v>1169</v>
       </c>
       <c r="B537" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C537" t="s">
         <v>25</v>
@@ -29604,7 +29628,7 @@
         <v>1169</v>
       </c>
       <c r="B538" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C538" t="s">
         <v>33</v>
@@ -29642,7 +29666,7 @@
         <v>1169</v>
       </c>
       <c r="B539" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C539" t="s">
         <v>33</v>
@@ -29680,7 +29704,7 @@
         <v>1169</v>
       </c>
       <c r="B540" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C540" t="s">
         <v>25</v>
@@ -29718,7 +29742,7 @@
         <v>1169</v>
       </c>
       <c r="B541" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C541" t="s">
         <v>25</v>
@@ -29756,7 +29780,7 @@
         <v>1169</v>
       </c>
       <c r="B542" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C542" t="s">
         <v>25</v>
@@ -29794,7 +29818,7 @@
         <v>1169</v>
       </c>
       <c r="B543" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C543" t="s">
         <v>25</v>
@@ -29832,7 +29856,7 @@
         <v>1169</v>
       </c>
       <c r="B544" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C544" t="s">
         <v>25</v>
@@ -29870,7 +29894,7 @@
         <v>1169</v>
       </c>
       <c r="B545" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C545" t="s">
         <v>33</v>
@@ -29908,7 +29932,7 @@
         <v>1169</v>
       </c>
       <c r="B546" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C546" t="s">
         <v>33</v>
@@ -29946,7 +29970,7 @@
         <v>1169</v>
       </c>
       <c r="B547" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C547" t="s">
         <v>33</v>
@@ -29984,7 +30008,7 @@
         <v>1169</v>
       </c>
       <c r="B548" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C548" t="s">
         <v>33</v>
@@ -30022,7 +30046,7 @@
         <v>1169</v>
       </c>
       <c r="B549" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C549" t="s">
         <v>25</v>
@@ -30060,7 +30084,7 @@
         <v>1169</v>
       </c>
       <c r="B550" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C550" t="s">
         <v>25</v>
@@ -30098,7 +30122,7 @@
         <v>1169</v>
       </c>
       <c r="B551" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C551" t="s">
         <v>33</v>
@@ -30136,7 +30160,7 @@
         <v>1169</v>
       </c>
       <c r="B552" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C552" t="s">
         <v>25</v>
@@ -30174,7 +30198,7 @@
         <v>1169</v>
       </c>
       <c r="B553" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C553" t="s">
         <v>33</v>
@@ -30212,7 +30236,7 @@
         <v>1169</v>
       </c>
       <c r="B554" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C554" t="s">
         <v>111</v>
@@ -30250,7 +30274,7 @@
         <v>1169</v>
       </c>
       <c r="B555" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C555" t="s">
         <v>25</v>
@@ -30288,7 +30312,7 @@
         <v>1169</v>
       </c>
       <c r="B556" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C556" t="s">
         <v>25</v>
@@ -30326,7 +30350,7 @@
         <v>1169</v>
       </c>
       <c r="B557" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C557" t="s">
         <v>25</v>
@@ -30364,7 +30388,7 @@
         <v>1169</v>
       </c>
       <c r="B558" t="s">
-        <v>276</v>
+        <v>1375</v>
       </c>
       <c r="C558" t="s">
         <v>33</v>

</xml_diff>